<commit_message>
Audit fixes + updated labour rules
</commit_message>
<xml_diff>
--- a/00_Production_Source_Table.xlsx
+++ b/00_Production_Source_Table.xlsx
@@ -2285,7 +2285,11 @@
           <t>Reheat Beef Stroganoff (Sun Dinner)</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G10" s="7" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr">
         <is>
@@ -2359,7 +2363,11 @@
           <t>Reheat Vegan Mushroom Stroganoff (Sun Dinner — Veg)</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>12 lbs</t>
+        </is>
+      </c>
       <c r="G11" s="7" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr">
         <is>
@@ -2521,7 +2529,11 @@
           <t>HOT Beef Stroganoff → Dinner</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G13" s="15" t="inlineStr"/>
       <c r="H13" s="15" t="inlineStr">
         <is>
@@ -2595,7 +2607,11 @@
           <t>HOT Falafels → Lunch (Veg)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -2669,7 +2685,11 @@
           <t>Heat Falafel (frozen → oven) (Mon Lunch — Veg)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>40 pcs</t>
+        </is>
+      </c>
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr">
         <is>
@@ -3172,7 +3192,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G21" s="15" t="inlineStr"/>
       <c r="H21" s="15" t="inlineStr">
         <is>
@@ -3234,7 +3258,11 @@
           <t>HOT Jerk Chicken → Dinner</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr"/>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>1.5 hotels</t>
+        </is>
+      </c>
       <c r="G22" s="15" t="inlineStr"/>
       <c r="H22" s="15" t="inlineStr">
         <is>
@@ -3394,7 +3422,11 @@
           <t>HOT Beef Nacho Mix → Lunch</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr">
         <is>
@@ -3468,7 +3500,11 @@
           <t>HOT Vegan Nacho Mix → Lunch (Veg)</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr">
         <is>
@@ -3624,7 +3660,11 @@
           <t>Reheat Vegan Nacho Mix (Tue Lunch)</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr"/>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>15 lbs</t>
+        </is>
+      </c>
       <c r="G27" s="7" t="inlineStr"/>
       <c r="H27" s="7" t="inlineStr">
         <is>
@@ -4308,10 +4348,8 @@
           <t>Pork braise</t>
         </is>
       </c>
-      <c r="K35" s="7" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="K35" s="7" t="n">
+        <v>60</v>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
@@ -4392,10 +4430,8 @@
           <t>Pork braise</t>
         </is>
       </c>
-      <c r="K36" s="7" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="K36" s="7" t="n">
+        <v>60</v>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
@@ -4535,7 +4571,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F38" s="15" t="inlineStr"/>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G38" s="15" t="inlineStr"/>
       <c r="H38" s="15" t="inlineStr">
         <is>
@@ -4597,7 +4637,11 @@
           <t>HOT Pork/Chicken/Halal Carnitas → Dinner</t>
         </is>
       </c>
-      <c r="F39" s="15" t="inlineStr"/>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G39" s="15" t="inlineStr">
         <is>
           <t>5 oz</t>
@@ -4765,7 +4809,11 @@
           <t>HOT Crispy Chicken Tenders → Lunch</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -4839,7 +4887,11 @@
           <t>HOT Vegan Tenders → Lunch (Veg)</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr">
         <is>
@@ -4913,7 +4965,11 @@
           <t>Cold Chiffonade Lettuce &amp; Sliced Peppers → Lunch (wraps)</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>1 hotel</t>
+        </is>
+      </c>
       <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="3" t="inlineStr">
         <is>
@@ -4989,7 +5045,11 @@
           <t>Heat Crispy Chicken + Vegan Tenders (Wed Lunch)</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr"/>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>4.5 hotels</t>
+        </is>
+      </c>
       <c r="G44" s="7" t="inlineStr"/>
       <c r="H44" s="7" t="inlineStr">
         <is>
@@ -5063,7 +5123,11 @@
           <t>Cook Adobo Pork/Chicken</t>
         </is>
       </c>
-      <c r="F45" s="13" t="inlineStr"/>
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>40 lbs/32 lbs cooked</t>
+        </is>
+      </c>
       <c r="G45" s="13" t="inlineStr"/>
       <c r="H45" s="13" t="inlineStr">
         <is>
@@ -5642,7 +5706,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F52" s="15" t="inlineStr"/>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G52" s="15" t="inlineStr"/>
       <c r="H52" s="15" t="inlineStr">
         <is>
@@ -6195,10 +6263,8 @@
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr"/>
-      <c r="K59" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="K59" s="13" t="n">
+        <v>240</v>
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
@@ -6681,7 +6747,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F65" s="15" t="inlineStr"/>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G65" s="15" t="inlineStr"/>
       <c r="H65" s="15" t="inlineStr">
         <is>
@@ -7344,7 +7414,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F73" s="15" t="inlineStr"/>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G73" s="15" t="inlineStr"/>
       <c r="H73" s="15" t="inlineStr">
         <is>
@@ -7564,7 +7638,7 @@
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>2 hotels</t>
+          <t>3 hotels</t>
         </is>
       </c>
       <c r="G76" s="15" t="inlineStr"/>
@@ -7600,10 +7674,8 @@
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P76" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="P76" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="Q76" s="15" t="inlineStr">
         <is>
@@ -7728,7 +7800,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>1 hotel</t>
+          <t>0.5 hotel</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr"/>
@@ -7768,10 +7840,8 @@
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P78" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P78" s="3" t="n">
+        <v>0.5</v>
       </c>
       <c r="Q78" s="3" t="inlineStr">
         <is>
@@ -7810,7 +7880,11 @@
           <t>Reheat CONC Salad Beef + Vegan (Sat Lunch)</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr"/>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>80 lbs + 15 lbs</t>
+        </is>
+      </c>
       <c r="G79" s="7" t="inlineStr"/>
       <c r="H79" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8543,11 @@
           <t>Rice (Sat Dinner)</t>
         </is>
       </c>
-      <c r="F87" s="13" t="inlineStr"/>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G87" s="13" t="inlineStr"/>
       <c r="H87" s="13" t="inlineStr"/>
       <c r="I87" s="13" t="inlineStr">
@@ -8627,7 +8705,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F89" s="15" t="inlineStr"/>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G89" s="15" t="inlineStr"/>
       <c r="H89" s="15" t="inlineStr">
         <is>
@@ -8863,7 +8945,11 @@
           <t>HOT Carrot Cabbage Fry → Dinner side</t>
         </is>
       </c>
-      <c r="F92" s="15" t="inlineStr"/>
+      <c r="F92" s="15" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G92" s="15" t="inlineStr"/>
       <c r="H92" s="15" t="inlineStr">
         <is>
@@ -8943,7 +9029,11 @@
           <t>HOT Rice → Dinner</t>
         </is>
       </c>
-      <c r="F93" s="15" t="inlineStr"/>
+      <c r="F93" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G93" s="15" t="inlineStr"/>
       <c r="H93" s="15" t="inlineStr"/>
       <c r="I93" s="15" t="inlineStr">
@@ -8977,10 +9067,8 @@
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P93" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P93" s="15" t="n">
+        <v>4</v>
       </c>
       <c r="Q93" s="15" t="inlineStr">
         <is>
@@ -10061,7 +10149,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G12" s="15" t="inlineStr"/>
       <c r="H12" s="15" t="inlineStr">
         <is>
@@ -11404,7 +11496,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr"/>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G28" s="15" t="inlineStr"/>
       <c r="H28" s="15" t="inlineStr">
         <is>
@@ -11640,7 +11736,11 @@
           <t>HOT Rice → Dinner</t>
         </is>
       </c>
-      <c r="F31" s="15" t="inlineStr"/>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G31" s="15" t="inlineStr"/>
       <c r="H31" s="15" t="inlineStr">
         <is>
@@ -11714,7 +11814,11 @@
           <t>HOT Green Beans → Dinner side</t>
         </is>
       </c>
-      <c r="F32" s="15" t="inlineStr"/>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G32" s="15" t="inlineStr"/>
       <c r="H32" s="15" t="inlineStr">
         <is>
@@ -12532,7 +12636,11 @@
           <t>Steam Broccoli (Tue Dinner side)</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr"/>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G42" s="13" t="inlineStr"/>
       <c r="H42" s="13" t="inlineStr">
         <is>
@@ -12684,7 +12792,11 @@
           <t>HOT Steamed Rice → Dinner</t>
         </is>
       </c>
-      <c r="F44" s="15" t="inlineStr"/>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G44" s="15" t="inlineStr"/>
       <c r="H44" s="15" t="inlineStr">
         <is>
@@ -12758,7 +12870,11 @@
           <t>HOT Broccoli → Dinner side</t>
         </is>
       </c>
-      <c r="F45" s="15" t="inlineStr"/>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G45" s="15" t="inlineStr"/>
       <c r="H45" s="15" t="inlineStr">
         <is>
@@ -13849,7 +13965,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F58" s="15" t="inlineStr"/>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G58" s="15" t="inlineStr"/>
       <c r="H58" s="15" t="inlineStr">
         <is>
@@ -14087,7 +14207,11 @@
           <t>HOT Coconut Rice &amp; Peas → Dinner</t>
         </is>
       </c>
-      <c r="F61" s="15" t="inlineStr"/>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G61" s="15" t="inlineStr"/>
       <c r="H61" s="15" t="inlineStr">
         <is>
@@ -14161,7 +14285,11 @@
           <t>HOT Eggplant/Cassava Stew → Dinner</t>
         </is>
       </c>
-      <c r="F62" s="15" t="inlineStr"/>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G62" s="15" t="inlineStr"/>
       <c r="H62" s="15" t="inlineStr">
         <is>
@@ -19138,7 +19266,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>50 pcs</t>
+          <t>2 hotels</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr"/>
@@ -19174,10 +19302,8 @@
           <t>LUNCH</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P17" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
@@ -19718,7 +19844,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F24" s="15" t="inlineStr"/>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G24" s="15" t="inlineStr"/>
       <c r="H24" s="15" t="inlineStr">
         <is>
@@ -21294,7 +21424,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F43" s="15" t="inlineStr"/>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G43" s="15" t="inlineStr"/>
       <c r="H43" s="15" t="inlineStr">
         <is>
@@ -21704,7 +21838,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>155 pcs</t>
+          <t>4 hotels</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr"/>
@@ -21740,10 +21874,8 @@
           <t>LUNCH</t>
         </is>
       </c>
-      <c r="P48" s="3" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="P48" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
@@ -21864,7 +21996,11 @@
           <t>Cold Chiffonade Lettuce &amp; Sliced Peppers → Lunch (wraps)</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>1 hotel</t>
+        </is>
+      </c>
       <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="3" t="inlineStr">
         <is>
@@ -22613,7 +22749,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F59" s="15" t="inlineStr"/>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G59" s="15" t="inlineStr"/>
       <c r="H59" s="15" t="inlineStr">
         <is>
@@ -23503,10 +23643,8 @@
           <t>Stove top</t>
         </is>
       </c>
-      <c r="K70" s="13" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
+      <c r="K70" s="13" t="n">
+        <v>240</v>
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
@@ -23981,7 +24119,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F76" s="15" t="inlineStr"/>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G76" s="15" t="inlineStr"/>
       <c r="H76" s="15" t="inlineStr">
         <is>
@@ -24045,7 +24187,7 @@
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>2.5 hotels</t>
+          <t>3 hotels</t>
         </is>
       </c>
       <c r="G77" s="15" t="inlineStr">
@@ -24209,7 +24351,11 @@
           <t>HOT Chakalaka → Dinner side</t>
         </is>
       </c>
-      <c r="F79" s="15" t="inlineStr"/>
+      <c r="F79" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G79" s="15" t="inlineStr"/>
       <c r="H79" s="15" t="inlineStr">
         <is>
@@ -24369,7 +24515,11 @@
           <t>White Chilli Chicken Pasta (→ Wk4 Sun Dinner)</t>
         </is>
       </c>
-      <c r="F81" s="13" t="inlineStr"/>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>100 lbs</t>
+        </is>
+      </c>
       <c r="G81" s="13" t="inlineStr"/>
       <c r="H81" s="13" t="inlineStr">
         <is>
@@ -24935,7 +25085,11 @@
           <t>HOT Vegan/No-Soy Mushroom Fried Rice → Dinner (Veg)</t>
         </is>
       </c>
-      <c r="F88" s="15" t="inlineStr"/>
+      <c r="F88" s="15" t="inlineStr">
+        <is>
+          <t>1 hotel</t>
+        </is>
+      </c>
       <c r="G88" s="15" t="inlineStr"/>
       <c r="H88" s="15" t="inlineStr"/>
       <c r="I88" s="15" t="inlineStr">
@@ -25011,7 +25165,11 @@
           <t>HOT Spring Rolls → Dinner side</t>
         </is>
       </c>
-      <c r="F89" s="15" t="inlineStr"/>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G89" s="15" t="inlineStr"/>
       <c r="H89" s="15" t="inlineStr"/>
       <c r="I89" s="15" t="inlineStr">
@@ -26180,7 +26338,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F103" s="15" t="inlineStr"/>
+      <c r="F103" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G103" s="15" t="inlineStr"/>
       <c r="H103" s="15" t="inlineStr">
         <is>
@@ -26242,7 +26404,11 @@
           <t>Pick up Pepperoni + Veg Pizza at vendor</t>
         </is>
       </c>
-      <c r="F104" s="15" t="inlineStr"/>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G104" s="15" t="inlineStr"/>
       <c r="H104" s="15" t="inlineStr">
         <is>
@@ -26404,7 +26570,11 @@
           <t>HOT Potato Wedges → Dinner</t>
         </is>
       </c>
-      <c r="F106" s="15" t="inlineStr"/>
+      <c r="F106" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G106" s="15" t="inlineStr">
         <is>
           <t>6 oz</t>
@@ -26849,10 +27019,8 @@
       </c>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
+      <c r="P4" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -27399,7 +27567,11 @@
           <t>Reheat White Chilli Chicken Pasta (Sun Dinner)</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>80 lbs</t>
+        </is>
+      </c>
       <c r="G11" s="7" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr">
         <is>
@@ -27901,7 +28073,11 @@
           <t>HOT Pasta + Broccoli &amp; Carrot → Dinner</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>9 hotels</t>
+        </is>
+      </c>
       <c r="G17" s="15" t="inlineStr"/>
       <c r="H17" s="15" t="inlineStr">
         <is>
@@ -28166,10 +28342,8 @@
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr"/>
-      <c r="K20" s="13" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
+      <c r="K20" s="13" t="n">
+        <v>60</v>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
@@ -28968,7 +29142,11 @@
           <t>HOT Curry Fish → Dinner</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr"/>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G30" s="15" t="inlineStr"/>
       <c r="H30" s="15" t="inlineStr"/>
       <c r="I30" s="15" t="inlineStr">
@@ -29042,7 +29220,11 @@
           <t>HOT Curry Spiced Tofu → Dinner (Veg)</t>
         </is>
       </c>
-      <c r="F31" s="15" t="inlineStr"/>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G31" s="15" t="inlineStr"/>
       <c r="H31" s="15" t="inlineStr"/>
       <c r="I31" s="15" t="inlineStr">
@@ -29116,7 +29298,11 @@
           <t>HOT Green Curry Sauce → Dinner</t>
         </is>
       </c>
-      <c r="F32" s="15" t="inlineStr"/>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G32" s="15" t="inlineStr"/>
       <c r="H32" s="15" t="inlineStr"/>
       <c r="I32" s="15" t="inlineStr">
@@ -29192,7 +29378,11 @@
           <t>HOT Rice + Green Beans → Dinner</t>
         </is>
       </c>
-      <c r="F33" s="15" t="inlineStr"/>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>7 hotels</t>
+        </is>
+      </c>
       <c r="G33" s="15" t="inlineStr"/>
       <c r="H33" s="15" t="inlineStr">
         <is>
@@ -30831,7 +31021,11 @@
           <t>HOT BBQ Chicken Legs → Dinner</t>
         </is>
       </c>
-      <c r="F53" s="15" t="inlineStr"/>
+      <c r="F53" s="15" t="inlineStr">
+        <is>
+          <t>1 hotel</t>
+        </is>
+      </c>
       <c r="G53" s="15" t="inlineStr"/>
       <c r="H53" s="15" t="inlineStr"/>
       <c r="I53" s="15" t="inlineStr">
@@ -30907,7 +31101,11 @@
           <t>HOT BBQ Vegan Tenders → Dinner (Veg)</t>
         </is>
       </c>
-      <c r="F54" s="15" t="inlineStr"/>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G54" s="15" t="inlineStr"/>
       <c r="H54" s="15" t="inlineStr"/>
       <c r="I54" s="15" t="inlineStr">
@@ -30983,7 +31181,11 @@
           <t>HOT Herb Garlic Potatoes → Dinner</t>
         </is>
       </c>
-      <c r="F55" s="15" t="inlineStr"/>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G55" s="15" t="inlineStr"/>
       <c r="H55" s="15" t="inlineStr"/>
       <c r="I55" s="15" t="inlineStr">
@@ -31059,7 +31261,11 @@
           <t>HOT Peas &amp; Carrot → Dinner side</t>
         </is>
       </c>
-      <c r="F56" s="15" t="inlineStr"/>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G56" s="15" t="inlineStr"/>
       <c r="H56" s="15" t="inlineStr"/>
       <c r="I56" s="15" t="inlineStr">
@@ -32241,7 +32447,11 @@
           <t>HOT Eggplant/Cassava Stew → Dinner</t>
         </is>
       </c>
-      <c r="F70" s="15" t="inlineStr"/>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>2 hotels</t>
+        </is>
+      </c>
       <c r="G70" s="15" t="inlineStr"/>
       <c r="H70" s="15" t="inlineStr">
         <is>
@@ -32315,7 +32525,11 @@
           <t>HOT Beef &amp; Vegetable Stew → Dinner</t>
         </is>
       </c>
-      <c r="F71" s="15" t="inlineStr"/>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G71" s="15" t="inlineStr"/>
       <c r="H71" s="15" t="inlineStr"/>
       <c r="I71" s="15" t="inlineStr">
@@ -32463,7 +32677,11 @@
           <t>HOT Halal Beef Burgers → Lunch</t>
         </is>
       </c>
-      <c r="F73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="3" t="inlineStr">
         <is>
@@ -33591,7 +33809,11 @@
           <t>HOT Chow Mein + Nappa Cabbage → Dinner</t>
         </is>
       </c>
-      <c r="F87" s="15" t="inlineStr"/>
+      <c r="F87" s="15" t="inlineStr">
+        <is>
+          <t>8 hotels</t>
+        </is>
+      </c>
       <c r="G87" s="15" t="inlineStr"/>
       <c r="H87" s="15" t="inlineStr">
         <is>
@@ -33873,10 +34095,8 @@
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P90" s="15" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="P90" s="15" t="n">
+        <v>4</v>
       </c>
       <c r="Q90" s="15" t="inlineStr">
         <is>
@@ -33917,7 +34137,7 @@
       </c>
       <c r="F91" s="15" t="inlineStr">
         <is>
-          <t>0.5 unit</t>
+          <t>2 bins</t>
         </is>
       </c>
       <c r="G91" s="15" t="inlineStr"/>
@@ -33925,7 +34145,7 @@
       <c r="I91" s="15" t="inlineStr"/>
       <c r="J91" s="16" t="inlineStr">
         <is>
-          <t>LAN → Rex</t>
+          <t>⚠ CONFIRM 2 bins/4u — LAN → Rex</t>
         </is>
       </c>
       <c r="K91" s="15" t="inlineStr"/>
@@ -33946,7 +34166,7 @@
         </is>
       </c>
       <c r="P91" s="18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q91" s="15" t="inlineStr">
         <is>
@@ -34791,7 +35011,11 @@
           <t>HOT Tandoori Tofu → Dinner (Veg)</t>
         </is>
       </c>
-      <c r="F102" s="15" t="inlineStr"/>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G102" s="15" t="inlineStr"/>
       <c r="H102" s="15" t="inlineStr"/>
       <c r="I102" s="15" t="inlineStr">
@@ -34865,7 +35089,11 @@
           <t>Pick up Baked Rolls at GC</t>
         </is>
       </c>
-      <c r="F103" s="15" t="inlineStr"/>
+      <c r="F103" s="15" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
       <c r="G103" s="15" t="inlineStr"/>
       <c r="H103" s="15" t="inlineStr"/>
       <c r="I103" s="15" t="inlineStr"/>
@@ -35661,7 +35889,11 @@
           <t>Rice (Sat Dinner)</t>
         </is>
       </c>
-      <c r="F113" s="13" t="inlineStr"/>
+      <c r="F113" s="13" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G113" s="13" t="inlineStr"/>
       <c r="H113" s="13" t="inlineStr">
         <is>
@@ -35737,7 +35969,11 @@
           <t>HOT Beef Massaman Curry → Dinner</t>
         </is>
       </c>
-      <c r="F114" s="15" t="inlineStr"/>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G114" s="15" t="inlineStr"/>
       <c r="H114" s="15" t="inlineStr"/>
       <c r="I114" s="15" t="inlineStr">
@@ -35811,7 +36047,11 @@
           <t>HOT Vegan Massaman Curry → Dinner (Veg)</t>
         </is>
       </c>
-      <c r="F115" s="15" t="inlineStr"/>
+      <c r="F115" s="15" t="inlineStr">
+        <is>
+          <t>0.5 hotels</t>
+        </is>
+      </c>
       <c r="G115" s="15" t="inlineStr"/>
       <c r="H115" s="15" t="inlineStr"/>
       <c r="I115" s="15" t="inlineStr">
@@ -35885,7 +36125,11 @@
           <t>HOT Rice → Dinner side</t>
         </is>
       </c>
-      <c r="F116" s="15" t="inlineStr"/>
+      <c r="F116" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
       <c r="G116" s="15" t="inlineStr"/>
       <c r="H116" s="15" t="inlineStr">
         <is>
@@ -35959,7 +36203,11 @@
           <t>Cold Broccoli Salad → NC Wk1 Sun Lunch</t>
         </is>
       </c>
-      <c r="F117" s="15" t="inlineStr"/>
+      <c r="F117" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
       <c r="G117" s="15" t="inlineStr"/>
       <c r="H117" s="15" t="inlineStr"/>
       <c r="I117" s="15" t="inlineStr">

</xml_diff>

<commit_message>
PROD/COOK updates and Browser cache defeating
</commit_message>
<xml_diff>
--- a/00_Production_Source_Table.xlsx
+++ b/00_Production_Source_Table.xlsx
@@ -4375,7 +4375,7 @@
       <c r="Q35" s="7" t="inlineStr"/>
       <c r="R35" s="8" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Thu/Fri Production (prev. cycle)</t>
+          <t>Produced: Wk. 4 Saturday Production (prev. cycle)</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
       <c r="Q36" s="7" t="inlineStr"/>
       <c r="R36" s="8" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Thu/Fri Production (prev. cycle)</t>
+          <t>Produced: Wk. 4 Saturday Production (prev. cycle)</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="R39" s="16" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Thu/Fri Production (prev. cycle)</t>
+          <t>Produced: Wk. 4 Saturday Production (prev. cycle)</t>
         </is>
       </c>
     </row>
@@ -27488,7 +27488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T124"/>
+  <dimension ref="A1:T126"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -34252,58 +34252,68 @@
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>Carnitas Sauce (→ Wk. 1 Tues. Dinner)</t>
+          <t>Tuna Rex Salad Mix (→ Sat Lunch — make day before)</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>2 bins</t>
         </is>
       </c>
       <c r="G83" s="9" t="inlineStr"/>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>cambro</t>
-        </is>
-      </c>
-      <c r="I83" s="9" t="inlineStr"/>
-      <c r="J83" s="10" t="inlineStr"/>
+          <t>bus bin</t>
+        </is>
+      </c>
+      <c r="I83" s="9" t="inlineStr">
+        <is>
+          <t>2 bins</t>
+        </is>
+      </c>
+      <c r="J83" s="10" t="inlineStr">
+        <is>
+          <t>⚠ NO RECIPE | Mix; chill; send cold day-of</t>
+        </is>
+      </c>
       <c r="K83" s="9" t="inlineStr">
         <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L83" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="L83" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
         </is>
       </c>
       <c r="M83" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N83" s="9" t="inlineStr">
         <is>
-          <t>TUESDAY</t>
+          <t>SATURDAY</t>
         </is>
       </c>
       <c r="O83" s="9" t="inlineStr">
         <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P83" s="9" t="n">
-        <v>1</v>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P83" s="9" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="Q83" s="9" t="inlineStr"/>
       <c r="R83" s="10" t="inlineStr">
         <is>
-          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
-        </is>
-      </c>
-      <c r="S83" s="12" t="n">
-        <v>5</v>
+          <t>Serves: Wk.4 Saturday Lunch</t>
+        </is>
+      </c>
+      <c r="S83" s="11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -34329,12 +34339,12 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>Season Carnitas Chicken (→ Wk. 1 Tues. Dinner)</t>
+          <t>Chickpea Rex Salad (→ Sat Lunch — make day before)</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>1 cs</t>
+          <t>3 bins</t>
         </is>
       </c>
       <c r="G84" s="9" t="inlineStr"/>
@@ -34345,48 +34355,50 @@
       </c>
       <c r="I84" s="9" t="inlineStr">
         <is>
-          <t>1 bin</t>
-        </is>
-      </c>
-      <c r="J84" s="10" t="inlineStr"/>
+          <t>3 bins</t>
+        </is>
+      </c>
+      <c r="J84" s="10" t="inlineStr">
+        <is>
+          <t>⚠ NO RECIPE | Dress; chill; send cold</t>
+        </is>
+      </c>
       <c r="K84" s="9" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L84" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L84" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
         </is>
       </c>
       <c r="M84" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N84" s="9" t="inlineStr">
         <is>
-          <t>TUESDAY</t>
+          <t>SATURDAY</t>
         </is>
       </c>
       <c r="O84" s="9" t="inlineStr">
         <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P84" s="9" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P84" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="Q84" s="9" t="inlineStr"/>
       <c r="R84" s="10" t="inlineStr">
         <is>
-          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
-        </is>
-      </c>
-      <c r="S84" s="12" t="n">
-        <v>5</v>
+          <t>Serves: Wk.4 Saturday Lunch</t>
+        </is>
+      </c>
+      <c r="S84" s="11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -34397,7 +34409,7 @@
       </c>
       <c r="B85" s="9" t="inlineStr">
         <is>
-          <t>THURSDAY</t>
+          <t>WEDNESDAY</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
@@ -34412,12 +34424,12 @@
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>Season Carnitas Pork (→ Wk. 1 Tues. Dinner)</t>
+          <t>Prep Slaw (→ Fri Lunch)</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>1 cs</t>
+          <t>???</t>
         </is>
       </c>
       <c r="G85" s="9" t="inlineStr"/>
@@ -34426,454 +34438,441 @@
           <t>bus bin</t>
         </is>
       </c>
-      <c r="I85" s="9" t="inlineStr">
-        <is>
-          <t>1 bin</t>
-        </is>
-      </c>
-      <c r="J85" s="10" t="inlineStr"/>
+      <c r="I85" s="9" t="inlineStr"/>
+      <c r="J85" s="10" t="inlineStr">
+        <is>
+          <t>Shred; dress; chill; send Thu PM</t>
+        </is>
+      </c>
       <c r="K85" s="9" t="inlineStr">
         <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="L85" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="L85" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
         </is>
       </c>
       <c r="M85" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N85" s="9" t="inlineStr">
         <is>
-          <t>TUESDAY</t>
+          <t>FRIDAY</t>
         </is>
       </c>
       <c r="O85" s="9" t="inlineStr">
         <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P85" s="9" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P85" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="Q85" s="9" t="inlineStr"/>
       <c r="R85" s="10" t="inlineStr">
         <is>
-          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
-        </is>
-      </c>
-      <c r="S85" s="12" t="n">
-        <v>5</v>
+          <t>Serves: Wk.4 Friday Lunch</t>
+        </is>
+      </c>
+      <c r="S85" s="11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="9" t="inlineStr">
+      <c r="A86" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B86" s="9" t="inlineStr">
+      <c r="B86" s="13" t="inlineStr">
         <is>
           <t>THURSDAY</t>
         </is>
       </c>
-      <c r="C86" s="9" t="inlineStr">
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="D86" s="13" t="inlineStr">
+        <is>
+          <t>COOK</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>Teriyaki Chicken Legs (Thu Dinner)</t>
+        </is>
+      </c>
+      <c r="F86" s="13" t="inlineStr">
+        <is>
+          <t>5 hotels</t>
+        </is>
+      </c>
+      <c r="G86" s="13" t="inlineStr"/>
+      <c r="H86" s="13" t="inlineStr"/>
+      <c r="I86" s="13" t="inlineStr"/>
+      <c r="J86" s="14" t="inlineStr">
+        <is>
+          <t>Combi roast</t>
+        </is>
+      </c>
+      <c r="K86" s="13" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M86" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N86" s="13" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="O86" s="13" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P86" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q86" s="13" t="inlineStr"/>
+      <c r="R86" s="14" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 4 Thursday Dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>COOK</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>Chow Mein + Nappa Cabbage (Thu Dinner side)</t>
+        </is>
+      </c>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>6 hotels</t>
+        </is>
+      </c>
+      <c r="G87" s="13" t="inlineStr"/>
+      <c r="H87" s="13" t="inlineStr"/>
+      <c r="I87" s="13" t="inlineStr"/>
+      <c r="J87" s="14" t="inlineStr">
+        <is>
+          <t>Wok/oven</t>
+        </is>
+      </c>
+      <c r="K87" s="13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M87" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N87" s="13" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="O87" s="13" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P87" s="13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Q87" s="13" t="inlineStr"/>
+      <c r="R87" s="14" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 4 Thursday Dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="C88" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>HOT Teriyaki Chicken + Five-Spice Tofu → Dinner</t>
+        </is>
+      </c>
+      <c r="F88" s="15" t="inlineStr">
+        <is>
+          <t>215 pcs</t>
+        </is>
+      </c>
+      <c r="G88" s="15" t="inlineStr"/>
+      <c r="H88" s="15" t="inlineStr">
+        <is>
+          <t>hotel/vac</t>
+        </is>
+      </c>
+      <c r="I88" s="15" t="inlineStr">
+        <is>
+          <t>6 hotels</t>
+        </is>
+      </c>
+      <c r="J88" s="16" t="inlineStr">
+        <is>
+          <t>Bloor → Rex</t>
+        </is>
+      </c>
+      <c r="K88" s="15" t="inlineStr"/>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M88" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N88" s="15" t="inlineStr"/>
+      <c r="O88" s="15" t="inlineStr"/>
+      <c r="P88" s="15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Q88" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R88" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk. 4 Tue (seasoned) → cooked Thu</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="C89" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>HOT Chow Mein + Nappa Cabbage → Dinner</t>
+        </is>
+      </c>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>8 hotels</t>
+        </is>
+      </c>
+      <c r="G89" s="15" t="inlineStr"/>
+      <c r="H89" s="15" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="I89" s="15" t="inlineStr">
+        <is>
+          <t>8 hotels</t>
+        </is>
+      </c>
+      <c r="J89" s="16" t="inlineStr">
+        <is>
+          <t>Bloor → Rex</t>
+        </is>
+      </c>
+      <c r="K89" s="15" t="inlineStr"/>
+      <c r="L89" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M89" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N89" s="15" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="O89" s="15" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P89" s="15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q89" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R89" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk. 4 Thursday Dinner (LAN same day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>THURSDAY</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>Cold Beef Nacho Mix → Rex fridge</t>
+        </is>
+      </c>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>80 lbs</t>
+        </is>
+      </c>
+      <c r="G90" s="15" t="inlineStr"/>
+      <c r="H90" s="15" t="inlineStr">
+        <is>
+          <t>vac</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>2u</t>
+        </is>
+      </c>
+      <c r="J90" s="16" t="inlineStr">
+        <is>
+          <t>Bloor → Rex; Rex holds until Wk1 Mon AM pull</t>
+        </is>
+      </c>
+      <c r="K90" s="15" t="inlineStr"/>
+      <c r="L90" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M90" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N90" s="15" t="inlineStr">
+        <is>
+          <t>WEDNESDAY</t>
+        </is>
+      </c>
+      <c r="O90" s="15" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="D86" s="9" t="inlineStr">
-        <is>
-          <t>PREP</t>
-        </is>
-      </c>
-      <c r="E86" s="10" t="inlineStr">
-        <is>
-          <t>Tuna Rex Salad Mix (→ Sat Lunch — make day before)</t>
-        </is>
-      </c>
-      <c r="F86" s="9" t="inlineStr">
-        <is>
-          <t>2 bins</t>
-        </is>
-      </c>
-      <c r="G86" s="9" t="inlineStr"/>
-      <c r="H86" s="9" t="inlineStr">
-        <is>
-          <t>bus bin</t>
-        </is>
-      </c>
-      <c r="I86" s="9" t="inlineStr">
-        <is>
-          <t>2 bins</t>
-        </is>
-      </c>
-      <c r="J86" s="10" t="inlineStr">
-        <is>
-          <t>⚠ NO RECIPE | Mix; chill; send cold day-of</t>
-        </is>
-      </c>
-      <c r="K86" s="9" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="L86" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
-        </is>
-      </c>
-      <c r="M86" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N86" s="9" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="O86" s="9" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="P86" s="9" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q86" s="9" t="inlineStr"/>
-      <c r="R86" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk.4 Saturday Lunch</t>
-        </is>
-      </c>
-      <c r="S86" s="11" t="n">
+      <c r="P90" s="17" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B87" s="9" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D87" s="9" t="inlineStr">
-        <is>
-          <t>PREP</t>
-        </is>
-      </c>
-      <c r="E87" s="10" t="inlineStr">
-        <is>
-          <t>Chickpea Rex Salad (→ Sat Lunch — make day before)</t>
-        </is>
-      </c>
-      <c r="F87" s="9" t="inlineStr">
-        <is>
-          <t>3 bins</t>
-        </is>
-      </c>
-      <c r="G87" s="9" t="inlineStr"/>
-      <c r="H87" s="9" t="inlineStr">
-        <is>
-          <t>bus bin</t>
-        </is>
-      </c>
-      <c r="I87" s="9" t="inlineStr">
-        <is>
-          <t>3 bins</t>
-        </is>
-      </c>
-      <c r="J87" s="10" t="inlineStr">
-        <is>
-          <t>⚠ NO RECIPE | Dress; chill; send cold</t>
-        </is>
-      </c>
-      <c r="K87" s="9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L87" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
-        </is>
-      </c>
-      <c r="M87" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N87" s="9" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="O87" s="9" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="P87" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q87" s="9" t="inlineStr"/>
-      <c r="R87" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk.4 Saturday Lunch</t>
-        </is>
-      </c>
-      <c r="S87" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B88" s="9" t="inlineStr">
-        <is>
-          <t>WEDNESDAY</t>
-        </is>
-      </c>
-      <c r="C88" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D88" s="9" t="inlineStr">
-        <is>
-          <t>PREP</t>
-        </is>
-      </c>
-      <c r="E88" s="10" t="inlineStr">
-        <is>
-          <t>Prep Slaw (→ Fri Lunch)</t>
-        </is>
-      </c>
-      <c r="F88" s="9" t="inlineStr">
-        <is>
-          <t>???</t>
-        </is>
-      </c>
-      <c r="G88" s="9" t="inlineStr"/>
-      <c r="H88" s="9" t="inlineStr">
-        <is>
-          <t>bus bin</t>
-        </is>
-      </c>
-      <c r="I88" s="9" t="inlineStr"/>
-      <c r="J88" s="10" t="inlineStr">
-        <is>
-          <t>Shred; dress; chill; send Thu PM</t>
-        </is>
-      </c>
-      <c r="K88" s="9" t="inlineStr">
-        <is>
-          <t>???</t>
-        </is>
-      </c>
-      <c r="L88" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
-        </is>
-      </c>
-      <c r="M88" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N88" s="9" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="O88" s="9" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="P88" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q88" s="9" t="inlineStr"/>
-      <c r="R88" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk.4 Friday Lunch</t>
-        </is>
-      </c>
-      <c r="S88" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C89" s="13" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="D89" s="13" t="inlineStr">
-        <is>
-          <t>COOK</t>
-        </is>
-      </c>
-      <c r="E89" s="14" t="inlineStr">
-        <is>
-          <t>Teriyaki Chicken Legs (Thu Dinner)</t>
-        </is>
-      </c>
-      <c r="F89" s="13" t="inlineStr">
-        <is>
-          <t>5 hotels</t>
-        </is>
-      </c>
-      <c r="G89" s="13" t="inlineStr"/>
-      <c r="H89" s="13" t="inlineStr"/>
-      <c r="I89" s="13" t="inlineStr"/>
-      <c r="J89" s="14" t="inlineStr">
-        <is>
-          <t>Combi roast</t>
-        </is>
-      </c>
-      <c r="K89" s="13" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="L89" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M89" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N89" s="13" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="O89" s="13" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P89" s="13" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="Q89" s="13" t="inlineStr"/>
-      <c r="R89" s="14" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 4 Thursday Dinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="D90" s="13" t="inlineStr">
-        <is>
-          <t>COOK</t>
-        </is>
-      </c>
-      <c r="E90" s="14" t="inlineStr">
-        <is>
-          <t>Chow Mein + Nappa Cabbage (Thu Dinner side)</t>
-        </is>
-      </c>
-      <c r="F90" s="13" t="inlineStr">
-        <is>
-          <t>6 hotels</t>
-        </is>
-      </c>
-      <c r="G90" s="13" t="inlineStr"/>
-      <c r="H90" s="13" t="inlineStr"/>
-      <c r="I90" s="13" t="inlineStr"/>
-      <c r="J90" s="14" t="inlineStr">
-        <is>
-          <t>Wok/oven</t>
-        </is>
-      </c>
-      <c r="K90" s="13" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="L90" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M90" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N90" s="13" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="O90" s="13" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P90" s="13" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Q90" s="13" t="inlineStr"/>
-      <c r="R90" s="14" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 4 Thursday Dinner</t>
+      <c r="Q90" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R90" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk. 4 Wednesday Production</t>
         </is>
       </c>
     </row>
@@ -34900,28 +34899,28 @@
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>HOT Teriyaki Chicken + Five-Spice Tofu → Dinner</t>
+          <t>Cold Vegan Nacho Mix → Rex fridge</t>
         </is>
       </c>
       <c r="F91" s="15" t="inlineStr">
         <is>
-          <t>215 pcs</t>
+          <t>15 lbs</t>
         </is>
       </c>
       <c r="G91" s="15" t="inlineStr"/>
       <c r="H91" s="15" t="inlineStr">
         <is>
-          <t>hotel/vac</t>
+          <t>vac</t>
         </is>
       </c>
       <c r="I91" s="15" t="inlineStr">
         <is>
-          <t>6 hotels</t>
+          <t>0.5u</t>
         </is>
       </c>
       <c r="J91" s="16" t="inlineStr">
         <is>
-          <t>Bloor → Rex</t>
+          <t>Bloor → Rex; Rex holds until Wk1 Mon AM pull</t>
         </is>
       </c>
       <c r="K91" s="15" t="inlineStr"/>
@@ -34935,12 +34934,18 @@
           <t>4</t>
         </is>
       </c>
-      <c r="N91" s="15" t="inlineStr"/>
-      <c r="O91" s="15" t="inlineStr"/>
-      <c r="P91" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="N91" s="15" t="inlineStr">
+        <is>
+          <t>WEDNESDAY</t>
+        </is>
+      </c>
+      <c r="O91" s="15" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="P91" s="17" t="n">
+        <v>0.5</v>
       </c>
       <c r="Q91" s="15" t="inlineStr">
         <is>
@@ -34949,7 +34954,7 @@
       </c>
       <c r="R91" s="16" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Tue (seasoned) → cooked Thu</t>
+          <t>Produced: Wk. 4 Wednesday Production</t>
         </is>
       </c>
     </row>
@@ -34976,34 +34981,34 @@
       </c>
       <c r="E92" s="16" t="inlineStr">
         <is>
-          <t>HOT Chow Mein + Nappa Cabbage → Dinner</t>
+          <t>Cold Chicken Ranch Mix → Fri Lunch</t>
         </is>
       </c>
       <c r="F92" s="15" t="inlineStr">
         <is>
-          <t>8 hotels</t>
+          <t>2 bins</t>
         </is>
       </c>
       <c r="G92" s="15" t="inlineStr"/>
       <c r="H92" s="15" t="inlineStr">
         <is>
-          <t>hotel</t>
+          <t>bus bin</t>
         </is>
       </c>
       <c r="I92" s="15" t="inlineStr">
         <is>
-          <t>8 hotels</t>
+          <t>2 bins</t>
         </is>
       </c>
       <c r="J92" s="16" t="inlineStr">
         <is>
-          <t>Bloor → Rex</t>
+          <t>LAN → Rex</t>
         </is>
       </c>
       <c r="K92" s="15" t="inlineStr"/>
-      <c r="L92" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
+      <c r="L92" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
         </is>
       </c>
       <c r="M92" s="15" t="inlineStr">
@@ -35011,20 +35016,14 @@
           <t>4</t>
         </is>
       </c>
-      <c r="N92" s="15" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
+      <c r="N92" s="15" t="inlineStr"/>
       <c r="O92" s="15" t="inlineStr">
         <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P92" s="15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="P92" s="15" t="n">
+        <v>4</v>
       </c>
       <c r="Q92" s="15" t="inlineStr">
         <is>
@@ -35033,7 +35032,7 @@
       </c>
       <c r="R92" s="16" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Thursday Dinner (LAN same day)</t>
+          <t>Produced: Wk.4 Wed Production (LAN)</t>
         </is>
       </c>
     </row>
@@ -35060,534 +35059,532 @@
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Cold Beef Nacho Mix → Rex fridge</t>
+          <t>Cold Slaw → Fri Lunch side</t>
         </is>
       </c>
       <c r="F93" s="15" t="inlineStr">
         <is>
-          <t>80 lbs</t>
+          <t>2 bins</t>
         </is>
       </c>
       <c r="G93" s="15" t="inlineStr"/>
-      <c r="H93" s="15" t="inlineStr">
+      <c r="H93" s="15" t="inlineStr"/>
+      <c r="I93" s="15" t="inlineStr"/>
+      <c r="J93" s="16" t="inlineStr">
+        <is>
+          <t>⚠ CONFIRM 2 bins/4u — LAN → Rex</t>
+        </is>
+      </c>
+      <c r="K93" s="15" t="inlineStr"/>
+      <c r="L93" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
+        </is>
+      </c>
+      <c r="M93" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N93" s="15" t="inlineStr"/>
+      <c r="O93" s="15" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="P93" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q93" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R93" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk.4 Wed Production (LAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>SEND AM</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>SEND AM</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>HOT Crispy Falafel → Lunch (Veg)</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>0.5 hotel</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>0.5 hotel</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>Bloor → Rex</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N94" s="3" t="inlineStr"/>
+      <c r="O94" s="3" t="inlineStr">
+        <is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P94" s="3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="Q94" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="R94" s="4" t="inlineStr">
+        <is>
+          <t>Produced: Wk.4 Fri Lunch (LAN same day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>HEAT</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Heat Falafel (frozen → oven) (Fri Lunch — Veg)</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>30 pcs</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr"/>
+      <c r="H95" s="7" t="inlineStr"/>
+      <c r="I95" s="7" t="inlineStr"/>
+      <c r="J95" s="8" t="inlineStr">
+        <is>
+          <t>Purchased frozen; heat day-of at Bloor</t>
+        </is>
+      </c>
+      <c r="K95" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L95" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M95" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N95" s="7" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="O95" s="7" t="inlineStr">
+        <is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P95" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q95" s="7" t="inlineStr"/>
+      <c r="R95" s="8" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 4 Friday Lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D96" s="13" t="inlineStr">
+        <is>
+          <t>COOK</t>
+        </is>
+      </c>
+      <c r="E96" s="14" t="inlineStr">
+        <is>
+          <t>Vegan Carnitas</t>
+        </is>
+      </c>
+      <c r="F96" s="13" t="inlineStr">
+        <is>
+          <t>15 lbs</t>
+        </is>
+      </c>
+      <c r="G96" s="13" t="inlineStr"/>
+      <c r="H96" s="13" t="inlineStr">
         <is>
           <t>vac</t>
         </is>
       </c>
-      <c r="I93" s="15" t="inlineStr">
-        <is>
-          <t>2u</t>
-        </is>
-      </c>
-      <c r="J93" s="16" t="inlineStr">
-        <is>
-          <t>Bloor → Rex; Rex holds until Wk1 Mon AM pull</t>
-        </is>
-      </c>
-      <c r="K93" s="15" t="inlineStr"/>
-      <c r="L93" s="5" t="inlineStr">
+      <c r="I96" s="13" t="inlineStr">
+        <is>
+          <t>1/2 hotel</t>
+        </is>
+      </c>
+      <c r="J96" s="14" t="inlineStr">
+        <is>
+          <t>Stove</t>
+        </is>
+      </c>
+      <c r="K96" s="13" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="L96" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M93" s="15" t="inlineStr">
+      <c r="M96" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N96" s="13" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O96" s="13" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P96" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q96" s="13" t="inlineStr"/>
+      <c r="R96" s="14" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S96" s="12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N93" s="15" t="inlineStr">
-        <is>
-          <t>WEDNESDAY</t>
-        </is>
-      </c>
-      <c r="O93" s="15" t="inlineStr">
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P93" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q93" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R93" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk. 4 Wednesday Production</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="15" t="inlineStr">
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr">
+        <is>
+          <t>Broccoli Prep (Saturday Lunch)</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>3 bins</t>
+        </is>
+      </c>
+      <c r="G97" s="9" t="inlineStr"/>
+      <c r="H97" s="9" t="inlineStr">
+        <is>
+          <t>bus bin</t>
+        </is>
+      </c>
+      <c r="I97" s="9" t="inlineStr">
+        <is>
+          <t>3 bins</t>
+        </is>
+      </c>
+      <c r="J97" s="10" t="inlineStr"/>
+      <c r="K97" s="9" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="L97" s="6" t="inlineStr">
+        <is>
+          <t>LAN</t>
+        </is>
+      </c>
+      <c r="M97" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B94" s="15" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C94" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="D94" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="E94" s="16" t="inlineStr">
-        <is>
-          <t>Cold Vegan Nacho Mix → Rex fridge</t>
-        </is>
-      </c>
-      <c r="F94" s="15" t="inlineStr">
-        <is>
-          <t>15 lbs</t>
-        </is>
-      </c>
-      <c r="G94" s="15" t="inlineStr"/>
-      <c r="H94" s="15" t="inlineStr">
-        <is>
-          <t>vac</t>
-        </is>
-      </c>
-      <c r="I94" s="15" t="inlineStr">
-        <is>
-          <t>0.5u</t>
-        </is>
-      </c>
-      <c r="J94" s="16" t="inlineStr">
-        <is>
-          <t>Bloor → Rex; Rex holds until Wk1 Mon AM pull</t>
-        </is>
-      </c>
-      <c r="K94" s="15" t="inlineStr"/>
-      <c r="L94" s="5" t="inlineStr">
+      <c r="N97" s="9" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="O97" s="9" t="inlineStr">
+        <is>
+          <t>LUNCH</t>
+        </is>
+      </c>
+      <c r="P97" s="9" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="Q97" s="9" t="inlineStr"/>
+      <c r="R97" s="10" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 4 Saturday Lunch</t>
+        </is>
+      </c>
+      <c r="S97" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>Prep Vegetable Biryani (→ Fri Dinner)</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="inlineStr">
+        <is>
+          <t>4 hotels veg</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr"/>
+      <c r="H98" s="9" t="inlineStr"/>
+      <c r="I98" s="9" t="inlineStr"/>
+      <c r="J98" s="10" t="inlineStr">
+        <is>
+          <t>⚠ NO RECIPE | Chop veg; hold for oven rice</t>
+        </is>
+      </c>
+      <c r="K98" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L98" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M94" s="15" t="inlineStr">
+      <c r="M98" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N94" s="15" t="inlineStr">
-        <is>
-          <t>WEDNESDAY</t>
-        </is>
-      </c>
-      <c r="O94" s="15" t="inlineStr">
+      <c r="N98" s="9" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="O98" s="9" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P98" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q98" s="9" t="inlineStr"/>
+      <c r="R98" s="10" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 4 Friday Dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P94" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q94" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R94" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk. 4 Wednesday Production</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B95" s="15" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C95" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="D95" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="E95" s="16" t="inlineStr">
-        <is>
-          <t>Cold Chicken Ranch Mix → Fri Lunch</t>
-        </is>
-      </c>
-      <c r="F95" s="15" t="inlineStr">
-        <is>
-          <t>2 bins</t>
-        </is>
-      </c>
-      <c r="G95" s="15" t="inlineStr"/>
-      <c r="H95" s="15" t="inlineStr">
-        <is>
-          <t>bus bin</t>
-        </is>
-      </c>
-      <c r="I95" s="15" t="inlineStr">
-        <is>
-          <t>2 bins</t>
-        </is>
-      </c>
-      <c r="J95" s="16" t="inlineStr">
-        <is>
-          <t>LAN → Rex</t>
-        </is>
-      </c>
-      <c r="K95" s="15" t="inlineStr"/>
-      <c r="L95" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
-        </is>
-      </c>
-      <c r="M95" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N95" s="15" t="inlineStr"/>
-      <c r="O95" s="15" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="P95" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q95" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R95" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk.4 Wed Production (LAN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B96" s="15" t="inlineStr">
-        <is>
-          <t>THURSDAY</t>
-        </is>
-      </c>
-      <c r="C96" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="D96" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="E96" s="16" t="inlineStr">
-        <is>
-          <t>Cold Slaw → Fri Lunch side</t>
-        </is>
-      </c>
-      <c r="F96" s="15" t="inlineStr">
-        <is>
-          <t>2 bins</t>
-        </is>
-      </c>
-      <c r="G96" s="15" t="inlineStr"/>
-      <c r="H96" s="15" t="inlineStr"/>
-      <c r="I96" s="15" t="inlineStr"/>
-      <c r="J96" s="16" t="inlineStr">
-        <is>
-          <t>⚠ CONFIRM 2 bins/4u — LAN → Rex</t>
-        </is>
-      </c>
-      <c r="K96" s="15" t="inlineStr"/>
-      <c r="L96" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
-        </is>
-      </c>
-      <c r="M96" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N96" s="15" t="inlineStr"/>
-      <c r="O96" s="15" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="P96" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q96" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R96" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk.4 Wed Production (LAN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>SEND AM</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>SEND AM</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>HOT Crispy Falafel → Lunch (Veg)</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t>0.5 hotel</t>
-        </is>
-      </c>
-      <c r="G97" s="3" t="inlineStr"/>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>hotel</t>
-        </is>
-      </c>
-      <c r="I97" s="3" t="inlineStr">
-        <is>
-          <t>0.5 hotel</t>
-        </is>
-      </c>
-      <c r="J97" s="4" t="inlineStr">
-        <is>
-          <t>Bloor → Rex</t>
-        </is>
-      </c>
-      <c r="K97" s="3" t="inlineStr"/>
-      <c r="L97" s="5" t="inlineStr">
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="E99" s="10" t="inlineStr">
+        <is>
+          <t>Jerk Marinade</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr"/>
+      <c r="H99" s="9" t="inlineStr">
+        <is>
+          <t>cambro/bag</t>
+        </is>
+      </c>
+      <c r="I99" s="9" t="inlineStr">
+        <is>
+          <t>1 bag/8 qt</t>
+        </is>
+      </c>
+      <c r="J99" s="10" t="inlineStr"/>
+      <c r="K99" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L99" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M97" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N97" s="3" t="inlineStr"/>
-      <c r="O97" s="3" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="P97" s="3" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="Q97" s="3" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="R97" s="4" t="inlineStr">
-        <is>
-          <t>Produced: Wk.4 Fri Lunch (LAN same day)</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>HEAT</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr">
-        <is>
-          <t>Heat Falafel (frozen → oven) (Fri Lunch — Veg)</t>
-        </is>
-      </c>
-      <c r="F98" s="7" t="inlineStr">
-        <is>
-          <t>30 pcs</t>
-        </is>
-      </c>
-      <c r="G98" s="7" t="inlineStr"/>
-      <c r="H98" s="7" t="inlineStr"/>
-      <c r="I98" s="7" t="inlineStr"/>
-      <c r="J98" s="8" t="inlineStr">
-        <is>
-          <t>Purchased frozen; heat day-of at Bloor</t>
-        </is>
-      </c>
-      <c r="K98" s="7" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L98" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M98" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="N98" s="7" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="O98" s="7" t="inlineStr">
-        <is>
-          <t>LUNCH</t>
-        </is>
-      </c>
-      <c r="P98" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q98" s="7" t="inlineStr"/>
-      <c r="R98" s="8" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 4 Friday Lunch</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B99" s="13" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="C99" s="13" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D99" s="13" t="inlineStr">
-        <is>
-          <t>COOK</t>
-        </is>
-      </c>
-      <c r="E99" s="14" t="inlineStr">
-        <is>
-          <t>Vegan Carnitas</t>
-        </is>
-      </c>
-      <c r="F99" s="13" t="inlineStr">
-        <is>
-          <t>15 lbs</t>
-        </is>
-      </c>
-      <c r="G99" s="13" t="inlineStr"/>
-      <c r="H99" s="13" t="inlineStr">
-        <is>
-          <t>vac</t>
-        </is>
-      </c>
-      <c r="I99" s="13" t="inlineStr">
-        <is>
-          <t>1/2 hotel</t>
-        </is>
-      </c>
-      <c r="J99" s="14" t="inlineStr">
-        <is>
-          <t>Stove</t>
-        </is>
-      </c>
-      <c r="K99" s="13" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="L99" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M99" s="13" t="inlineStr">
+      <c r="M99" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N99" s="13" t="inlineStr">
-        <is>
-          <t>TUESDAY</t>
-        </is>
-      </c>
-      <c r="O99" s="13" t="inlineStr">
+      <c r="N99" s="9" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="O99" s="9" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P99" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q99" s="13" t="inlineStr"/>
-      <c r="R99" s="14" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+      <c r="P99" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q99" s="9" t="inlineStr"/>
+      <c r="R99" s="10" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Monday Dinner</t>
         </is>
       </c>
       <c r="S99" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="100">
@@ -35613,12 +35610,12 @@
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>Broccoli Prep (Saturday Lunch)</t>
+          <t>Jerk Cauliflower</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>3 bins</t>
+          <t>15 pcs</t>
         </is>
       </c>
       <c r="G100" s="9" t="inlineStr"/>
@@ -35629,288 +35626,281 @@
       </c>
       <c r="I100" s="9" t="inlineStr">
         <is>
-          <t>3 bins</t>
+          <t>1/2 hotel</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr"/>
       <c r="K100" s="9" t="inlineStr">
         <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="L100" s="6" t="inlineStr">
-        <is>
-          <t>LAN</t>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
         </is>
       </c>
       <c r="M100" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N100" s="9" t="inlineStr">
         <is>
-          <t>SATURDAY</t>
+          <t>MONDAY</t>
         </is>
       </c>
       <c r="O100" s="9" t="inlineStr">
         <is>
-          <t>LUNCH</t>
+          <t>DINNER</t>
         </is>
       </c>
       <c r="P100" s="9" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q100" s="9" t="inlineStr"/>
       <c r="R100" s="10" t="inlineStr">
         <is>
-          <t>Serves: Wk. 4 Saturday Lunch</t>
-        </is>
-      </c>
-      <c r="S100" s="11" t="n">
+          <t>Serves: Wk. 1 Monday Dinner</t>
+        </is>
+      </c>
+      <c r="S100" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>FRIDAY</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Carnitas Sauce (→ Wk. 1 Tues. Dinner)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>cambro</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P101" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="9" t="inlineStr">
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S101" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B101" s="9" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>FRIDAY</t>
         </is>
       </c>
-      <c r="C101" s="9" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="D101" s="9" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>PREP</t>
         </is>
       </c>
-      <c r="E101" s="10" t="inlineStr">
-        <is>
-          <t>Prep Vegetable Biryani (→ Fri Dinner)</t>
-        </is>
-      </c>
-      <c r="F101" s="9" t="inlineStr">
-        <is>
-          <t>4 hotels veg</t>
-        </is>
-      </c>
-      <c r="G101" s="9" t="inlineStr"/>
-      <c r="H101" s="9" t="inlineStr"/>
-      <c r="I101" s="9" t="inlineStr"/>
-      <c r="J101" s="10" t="inlineStr">
-        <is>
-          <t>⚠ NO RECIPE | Chop veg; hold for oven rice</t>
-        </is>
-      </c>
-      <c r="K101" s="9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L101" s="5" t="inlineStr">
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Season Carnitas Chicken (→ Wk. 1 Tues. Dinner)</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>1 cs</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>bus bin</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>1 bin</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M101" s="9" t="inlineStr">
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S102" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N101" s="9" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>FRIDAY</t>
         </is>
       </c>
-      <c r="O101" s="9" t="inlineStr">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Season Carnitas Pork (→ Wk. 1 Tues. Dinner)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>1 cs</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>bus bin</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>1 bin</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P101" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q101" s="9" t="inlineStr"/>
-      <c r="R101" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 4 Friday Dinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B102" s="9" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="C102" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D102" s="9" t="inlineStr">
-        <is>
-          <t>PREP</t>
-        </is>
-      </c>
-      <c r="E102" s="10" t="inlineStr">
-        <is>
-          <t>Jerk Marinade</t>
-        </is>
-      </c>
-      <c r="F102" s="9" t="inlineStr">
-        <is>
-          <t>recipe</t>
-        </is>
-      </c>
-      <c r="G102" s="9" t="inlineStr"/>
-      <c r="H102" s="9" t="inlineStr">
-        <is>
-          <t>cambro/bag</t>
-        </is>
-      </c>
-      <c r="I102" s="9" t="inlineStr">
-        <is>
-          <t>1 bag/8 qt</t>
-        </is>
-      </c>
-      <c r="J102" s="10" t="inlineStr"/>
-      <c r="K102" s="9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L102" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M102" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N102" s="9" t="inlineStr">
-        <is>
-          <t>MONDAY</t>
-        </is>
-      </c>
-      <c r="O102" s="9" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P102" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q102" s="9" t="inlineStr"/>
-      <c r="R102" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 1 Monday Dinner</t>
-        </is>
-      </c>
-      <c r="S102" s="12" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B103" s="9" t="inlineStr">
-        <is>
-          <t>FRIDAY</t>
-        </is>
-      </c>
-      <c r="C103" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D103" s="9" t="inlineStr">
-        <is>
-          <t>PREP</t>
-        </is>
-      </c>
-      <c r="E103" s="10" t="inlineStr">
-        <is>
-          <t>Jerk Cauliflower</t>
-        </is>
-      </c>
-      <c r="F103" s="9" t="inlineStr">
-        <is>
-          <t>15 pcs</t>
-        </is>
-      </c>
-      <c r="G103" s="9" t="inlineStr"/>
-      <c r="H103" s="9" t="inlineStr">
-        <is>
-          <t>bus bin</t>
-        </is>
-      </c>
-      <c r="I103" s="9" t="inlineStr">
-        <is>
-          <t>1/2 hotel</t>
-        </is>
-      </c>
-      <c r="J103" s="10" t="inlineStr"/>
-      <c r="K103" s="9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="L103" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M103" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N103" s="9" t="inlineStr">
-        <is>
-          <t>MONDAY</t>
-        </is>
-      </c>
-      <c r="O103" s="9" t="inlineStr">
-        <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P103" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q103" s="9" t="inlineStr"/>
-      <c r="R103" s="10" t="inlineStr">
-        <is>
-          <t>Serves: Wk. 1 Monday Dinner</t>
-        </is>
-      </c>
-      <c r="S103" s="12" t="n">
-        <v>3</v>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S103" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="104">
@@ -36907,484 +36897,508 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="9" t="inlineStr">
+      <c r="A117" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B117" s="9" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="C117" s="9" t="inlineStr">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>COOK</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Cook Carnitas Pork (→ NC Wk1 Tue Dinner)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>1 cs</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>vac</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>1.5u</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Oven; cool then vac bag; hold Bloor fridge</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="D117" s="9" t="inlineStr">
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S117" t="n">
+        <v>3</v>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>COOK</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Cook Carnitas Chicken (→ NC Wk1 Tue Dinner)</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>1 cs</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>vac</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>1.0u</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Oven; cool then vac bag; hold Bloor fridge</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>TUESDAY</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Serves: Wk. 1 Tuesday Dinner (next cycle)</t>
+        </is>
+      </c>
+      <c r="S118" t="n">
+        <v>3</v>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>ALT</t>
         </is>
       </c>
-      <c r="E117" s="10" t="inlineStr">
+      <c r="E119" s="10" t="inlineStr">
         <is>
           <t>🔸 BLAND ALT — Plain Chicken Leg (3 pcs) + Naan + Stirfry Veg (NO PEANUTS) (Sat Dinner)</t>
         </is>
       </c>
-      <c r="F117" s="9" t="inlineStr">
+      <c r="F119" s="9" t="inlineStr">
         <is>
           <t>3 pcs</t>
         </is>
       </c>
-      <c r="G117" s="9" t="inlineStr">
+      <c r="G119" s="9" t="inlineStr">
         <is>
           <t>1 pc</t>
         </is>
       </c>
-      <c r="H117" s="9" t="inlineStr">
+      <c r="H119" s="9" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="I117" s="9" t="inlineStr"/>
-      <c r="J117" s="10" t="inlineStr">
+      <c r="I119" s="9" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
         <is>
           <t>For no-peanuts/no-nuts restrictions (2-3 ppl)</t>
         </is>
       </c>
-      <c r="K117" s="9" t="inlineStr">
+      <c r="K119" s="9" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L117" s="6" t="inlineStr">
+      <c r="L119" s="6" t="inlineStr">
         <is>
           <t>LAN</t>
         </is>
       </c>
-      <c r="M117" s="9" t="inlineStr">
+      <c r="M119" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N117" s="9" t="inlineStr">
+      <c r="N119" s="9" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="O117" s="9" t="inlineStr">
+      <c r="O119" s="9" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P117" s="9" t="n">
+      <c r="P119" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="Q117" s="9" t="inlineStr"/>
-      <c r="R117" s="10" t="inlineStr">
+      <c r="Q119" s="9" t="inlineStr"/>
+      <c r="R119" s="10" t="inlineStr">
         <is>
           <t>Serves: Wk. 4 Saturday Dinner</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="7" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B118" s="7" t="inlineStr">
+      <c r="B120" s="7" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="C118" s="7" t="inlineStr">
+      <c r="C120" s="7" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="D118" s="7" t="inlineStr">
+      <c r="D120" s="7" t="inlineStr">
         <is>
           <t>HEAT</t>
         </is>
       </c>
-      <c r="E118" s="8" t="inlineStr">
+      <c r="E120" s="8" t="inlineStr">
         <is>
           <t>Reheat Beef Massaman Curry (Sat Dinner)</t>
         </is>
       </c>
-      <c r="F118" s="7" t="inlineStr">
+      <c r="F120" s="7" t="inlineStr">
         <is>
           <t>110 lbs</t>
         </is>
       </c>
-      <c r="G118" s="7" t="inlineStr"/>
-      <c r="H118" s="7" t="inlineStr">
+      <c r="G120" s="7" t="inlineStr"/>
+      <c r="H120" s="7" t="inlineStr">
         <is>
           <t>vac</t>
         </is>
       </c>
-      <c r="I118" s="7" t="inlineStr">
+      <c r="I120" s="7" t="inlineStr">
         <is>
           <t>3u</t>
         </is>
       </c>
-      <c r="J118" s="8" t="inlineStr">
+      <c r="J120" s="8" t="inlineStr">
         <is>
           <t>Reheat bagged</t>
         </is>
       </c>
-      <c r="K118" s="7" t="inlineStr">
+      <c r="K120" s="7" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L118" s="5" t="inlineStr">
+      <c r="L120" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M118" s="7" t="inlineStr">
+      <c r="M120" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N118" s="7" t="inlineStr">
+      <c r="N120" s="7" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="O118" s="7" t="inlineStr">
+      <c r="O120" s="7" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P118" s="7" t="n">
+      <c r="P120" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="Q118" s="7" t="inlineStr"/>
-      <c r="R118" s="8" t="inlineStr">
+      <c r="Q120" s="7" t="inlineStr"/>
+      <c r="R120" s="8" t="inlineStr">
         <is>
           <t>Produced: Wk. 3 Saturday Production</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="7" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B119" s="7" t="inlineStr">
+      <c r="B121" s="7" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
+      <c r="C121" s="7" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="D119" s="7" t="inlineStr">
+      <c r="D121" s="7" t="inlineStr">
         <is>
           <t>HEAT</t>
         </is>
       </c>
-      <c r="E119" s="8" t="inlineStr">
+      <c r="E121" s="8" t="inlineStr">
         <is>
           <t>Reheat Vegan Massaman Curry (Sat Dinner — Veg)</t>
         </is>
       </c>
-      <c r="F119" s="7" t="inlineStr">
+      <c r="F121" s="7" t="inlineStr">
         <is>
           <t>15 lbs</t>
         </is>
       </c>
-      <c r="G119" s="7" t="inlineStr"/>
-      <c r="H119" s="7" t="inlineStr">
+      <c r="G121" s="7" t="inlineStr"/>
+      <c r="H121" s="7" t="inlineStr">
         <is>
           <t>vac</t>
         </is>
       </c>
-      <c r="I119" s="7" t="inlineStr">
+      <c r="I121" s="7" t="inlineStr">
         <is>
           <t>0.5u</t>
         </is>
       </c>
-      <c r="J119" s="8" t="inlineStr">
+      <c r="J121" s="8" t="inlineStr">
         <is>
           <t>Reheat bagged</t>
         </is>
       </c>
-      <c r="K119" s="7" t="inlineStr">
+      <c r="K121" s="7" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L119" s="5" t="inlineStr">
+      <c r="L121" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M119" s="7" t="inlineStr">
+      <c r="M121" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N119" s="7" t="inlineStr">
+      <c r="N121" s="7" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="O119" s="7" t="inlineStr">
+      <c r="O121" s="7" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P119" s="7" t="n">
+      <c r="P121" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q119" s="7" t="inlineStr"/>
-      <c r="R119" s="8" t="inlineStr">
+      <c r="Q121" s="7" t="inlineStr"/>
+      <c r="R121" s="8" t="inlineStr">
         <is>
           <t>Produced: Wk. 3 Saturday Production</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="13" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B120" s="13" t="inlineStr">
+      <c r="B122" s="13" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="C120" s="13" t="inlineStr">
+      <c r="C122" s="13" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="D120" s="13" t="inlineStr">
+      <c r="D122" s="13" t="inlineStr">
         <is>
           <t>COOK</t>
         </is>
       </c>
-      <c r="E120" s="14" t="inlineStr">
+      <c r="E122" s="14" t="inlineStr">
         <is>
           <t>Rice (Sat Dinner)</t>
         </is>
       </c>
-      <c r="F120" s="13" t="inlineStr">
+      <c r="F122" s="13" t="inlineStr">
         <is>
           <t>4 hotels</t>
         </is>
       </c>
-      <c r="G120" s="13" t="inlineStr"/>
-      <c r="H120" s="13" t="inlineStr">
+      <c r="G122" s="13" t="inlineStr"/>
+      <c r="H122" s="13" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="I120" s="13" t="inlineStr">
+      <c r="I122" s="13" t="inlineStr">
         <is>
           <t>1 hotel</t>
         </is>
       </c>
-      <c r="J120" s="14" t="inlineStr"/>
-      <c r="K120" s="13" t="inlineStr">
+      <c r="J122" s="14" t="inlineStr"/>
+      <c r="K122" s="13" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="L120" s="5" t="inlineStr">
+      <c r="L122" s="5" t="inlineStr">
         <is>
           <t>Bloor</t>
         </is>
       </c>
-      <c r="M120" s="13" t="inlineStr">
+      <c r="M122" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N120" s="13" t="inlineStr">
+      <c r="N122" s="13" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="O120" s="13" t="inlineStr">
+      <c r="O122" s="13" t="inlineStr">
         <is>
           <t>DINNER</t>
         </is>
       </c>
-      <c r="P120" s="13" t="inlineStr">
+      <c r="P122" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q120" s="13" t="inlineStr"/>
-      <c r="R120" s="14" t="inlineStr">
+      <c r="Q122" s="13" t="inlineStr"/>
+      <c r="R122" s="14" t="inlineStr">
         <is>
           <t>Serves: Wk. 4 Saturday Dinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B121" s="15" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="C121" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="D121" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="E121" s="16" t="inlineStr">
-        <is>
-          <t>HOT Beef Massaman Curry → Dinner</t>
-        </is>
-      </c>
-      <c r="F121" s="15" t="inlineStr">
-        <is>
-          <t>3 hotels</t>
-        </is>
-      </c>
-      <c r="G121" s="15" t="inlineStr"/>
-      <c r="H121" s="15" t="inlineStr"/>
-      <c r="I121" s="15" t="inlineStr">
-        <is>
-          <t>3u</t>
-        </is>
-      </c>
-      <c r="J121" s="16" t="inlineStr">
-        <is>
-          <t>Bloor → Rex</t>
-        </is>
-      </c>
-      <c r="K121" s="15" t="inlineStr"/>
-      <c r="L121" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M121" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="N121" s="15" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="O121" s="15" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="P121" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q121" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R121" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk. 3 Saturday Production</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B122" s="15" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="C122" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="D122" s="15" t="inlineStr">
-        <is>
-          <t>SEND PM</t>
-        </is>
-      </c>
-      <c r="E122" s="16" t="inlineStr">
-        <is>
-          <t>HOT Vegan Massaman Curry → Dinner (Veg)</t>
-        </is>
-      </c>
-      <c r="F122" s="15" t="inlineStr">
-        <is>
-          <t>0.5 hotels</t>
-        </is>
-      </c>
-      <c r="G122" s="15" t="inlineStr"/>
-      <c r="H122" s="15" t="inlineStr"/>
-      <c r="I122" s="15" t="inlineStr">
-        <is>
-          <t>0.5u</t>
-        </is>
-      </c>
-      <c r="J122" s="16" t="inlineStr">
-        <is>
-          <t>Bloor → Rex</t>
-        </is>
-      </c>
-      <c r="K122" s="15" t="inlineStr"/>
-      <c r="L122" s="5" t="inlineStr">
-        <is>
-          <t>Bloor</t>
-        </is>
-      </c>
-      <c r="M122" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="N122" s="15" t="inlineStr">
-        <is>
-          <t>SATURDAY</t>
-        </is>
-      </c>
-      <c r="O122" s="15" t="inlineStr">
-        <is>
-          <t>PRODUCTION</t>
-        </is>
-      </c>
-      <c r="P122" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q122" s="15" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="R122" s="16" t="inlineStr">
-        <is>
-          <t>Produced: Wk. 3 Saturday Production</t>
         </is>
       </c>
     </row>
@@ -37411,21 +37425,21 @@
       </c>
       <c r="E123" s="16" t="inlineStr">
         <is>
-          <t>HOT Rice → Dinner side</t>
+          <t>HOT Beef Massaman Curry → Dinner</t>
         </is>
       </c>
       <c r="F123" s="15" t="inlineStr">
         <is>
-          <t>4 hotels</t>
+          <t>3 hotels</t>
         </is>
       </c>
       <c r="G123" s="15" t="inlineStr"/>
-      <c r="H123" s="15" t="inlineStr">
-        <is>
-          <t>hotel</t>
-        </is>
-      </c>
-      <c r="I123" s="15" t="inlineStr"/>
+      <c r="H123" s="15" t="inlineStr"/>
+      <c r="I123" s="15" t="inlineStr">
+        <is>
+          <t>3u</t>
+        </is>
+      </c>
       <c r="J123" s="16" t="inlineStr">
         <is>
           <t>Bloor → Rex</t>
@@ -37439,7 +37453,7 @@
       </c>
       <c r="M123" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N123" s="15" t="inlineStr">
@@ -37449,11 +37463,11 @@
       </c>
       <c r="O123" s="15" t="inlineStr">
         <is>
-          <t>DINNER</t>
-        </is>
-      </c>
-      <c r="P123" s="26" t="n">
-        <v>4</v>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="P123" s="17" t="n">
+        <v>3</v>
       </c>
       <c r="Q123" s="15" t="inlineStr">
         <is>
@@ -37462,7 +37476,7 @@
       </c>
       <c r="R123" s="16" t="inlineStr">
         <is>
-          <t>Produced: Wk. 4 Saturday Dinner (same day)</t>
+          <t>Produced: Wk. 3 Saturday Production</t>
         </is>
       </c>
     </row>
@@ -37489,24 +37503,24 @@
       </c>
       <c r="E124" s="16" t="inlineStr">
         <is>
-          <t>Cold Broccoli Salad → NC Wk1 Sun Lunch</t>
+          <t>HOT Vegan Massaman Curry → Dinner (Veg)</t>
         </is>
       </c>
       <c r="F124" s="15" t="inlineStr">
         <is>
-          <t>3 hotels</t>
+          <t>0.5 hotels</t>
         </is>
       </c>
       <c r="G124" s="15" t="inlineStr"/>
       <c r="H124" s="15" t="inlineStr"/>
       <c r="I124" s="15" t="inlineStr">
         <is>
-          <t>3 hotels</t>
+          <t>0.5u</t>
         </is>
       </c>
       <c r="J124" s="16" t="inlineStr">
         <is>
-          <t>Bloor → Rex fridge</t>
+          <t>Bloor → Rex</t>
         </is>
       </c>
       <c r="K124" s="15" t="inlineStr"/>
@@ -37517,30 +37531,186 @@
       </c>
       <c r="M124" s="15" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N124" s="15" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="O124" s="15" t="inlineStr">
+        <is>
+          <t>PRODUCTION</t>
+        </is>
+      </c>
+      <c r="P124" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q124" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R124" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk. 3 Saturday Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N124" s="15" t="inlineStr">
+      <c r="B125" s="15" t="inlineStr">
         <is>
           <t>SATURDAY</t>
         </is>
       </c>
-      <c r="O124" s="15" t="inlineStr">
+      <c r="C125" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t>HOT Rice → Dinner side</t>
+        </is>
+      </c>
+      <c r="F125" s="15" t="inlineStr">
+        <is>
+          <t>4 hotels</t>
+        </is>
+      </c>
+      <c r="G125" s="15" t="inlineStr"/>
+      <c r="H125" s="15" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="I125" s="15" t="inlineStr"/>
+      <c r="J125" s="16" t="inlineStr">
+        <is>
+          <t>Bloor → Rex</t>
+        </is>
+      </c>
+      <c r="K125" s="15" t="inlineStr"/>
+      <c r="L125" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M125" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N125" s="15" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="O125" s="15" t="inlineStr">
+        <is>
+          <t>DINNER</t>
+        </is>
+      </c>
+      <c r="P125" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q125" s="15" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="R125" s="16" t="inlineStr">
+        <is>
+          <t>Produced: Wk. 4 Saturday Dinner (same day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="D126" s="15" t="inlineStr">
+        <is>
+          <t>SEND PM</t>
+        </is>
+      </c>
+      <c r="E126" s="16" t="inlineStr">
+        <is>
+          <t>Cold Broccoli Salad → NC Wk1 Sun Lunch</t>
+        </is>
+      </c>
+      <c r="F126" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
+      <c r="G126" s="15" t="inlineStr"/>
+      <c r="H126" s="15" t="inlineStr"/>
+      <c r="I126" s="15" t="inlineStr">
+        <is>
+          <t>3 hotels</t>
+        </is>
+      </c>
+      <c r="J126" s="16" t="inlineStr">
+        <is>
+          <t>Bloor → Rex fridge</t>
+        </is>
+      </c>
+      <c r="K126" s="15" t="inlineStr"/>
+      <c r="L126" s="5" t="inlineStr">
+        <is>
+          <t>Bloor</t>
+        </is>
+      </c>
+      <c r="M126" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N126" s="15" t="inlineStr">
+        <is>
+          <t>SATURDAY</t>
+        </is>
+      </c>
+      <c r="O126" s="15" t="inlineStr">
         <is>
           <t>PRODUCTION</t>
         </is>
       </c>
-      <c r="P124" s="15" t="inlineStr">
+      <c r="P126" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q124" s="15" t="inlineStr">
+      <c r="Q126" s="15" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="R124" s="16" t="inlineStr">
+      <c r="R126" s="16" t="inlineStr">
         <is>
           <t>Produced: Wk. 4 Saturday Production</t>
         </is>

</xml_diff>